<commit_message>
update: eficiencia nodo ciclo y global + actualización de plantilla
</commit_message>
<xml_diff>
--- a/plantilla_reporte.xlsx
+++ b/plantilla_reporte.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent>
     <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C3F31FD-E996-4CBD-A4DF-BBEAF3834610}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{228E5D52-D1FB-476C-85D0-790A8C4164C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="270" windowWidth="25440" windowHeight="15270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Simulación base" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="92">
   <si>
     <t>Corriente</t>
   </si>
@@ -140,9 +140,6 @@
     <t>Eficiencia Ciclo (%)</t>
   </si>
   <si>
-    <t>Eficiencia con ASU (%)</t>
-  </si>
-  <si>
     <t>Eficiencia Global CCS (%)</t>
   </si>
   <si>
@@ -159,9 +156,6 @@
   </si>
   <si>
     <t>eta_cycle (%)</t>
-  </si>
-  <si>
-    <t>eta_O2 (%)</t>
   </si>
   <si>
     <t>W_turb (MW)</t>
@@ -682,7 +676,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N25"/>
+  <dimension ref="A1:N24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29.28515625" bestFit="1" customWidth="1"/>
@@ -887,11 +881,6 @@
         <v>36</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>37</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -899,189 +888,185 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:BD1"/>
+  <dimension ref="A1:BC1"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AD1" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="AD1" s="1" t="s">
+      <c r="AE1" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="AE1" s="1" t="s">
+      <c r="AF1" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="AF1" s="1" t="s">
+      <c r="AG1" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="AG1" s="1" t="s">
+      <c r="AH1" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="AH1" s="1" t="s">
+      <c r="AI1" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="AI1" s="1" t="s">
+      <c r="AJ1" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="AJ1" s="1" t="s">
+      <c r="AK1" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="AK1" s="1" t="s">
+      <c r="AL1" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="AL1" s="1" t="s">
+      <c r="AM1" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="AM1" s="1" t="s">
+      <c r="AN1" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="AN1" s="1" t="s">
+      <c r="AO1" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="AO1" s="1" t="s">
+      <c r="AP1" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="AP1" s="1" t="s">
+      <c r="AQ1" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="AQ1" s="1" t="s">
+      <c r="AR1" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="AR1" s="1" t="s">
+      <c r="AS1" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="AS1" s="1" t="s">
+      <c r="AT1" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="AT1" s="1" t="s">
+      <c r="AU1" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="AU1" s="1" t="s">
+      <c r="AV1" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="AV1" s="1" t="s">
+      <c r="AW1" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="AW1" s="1" t="s">
+      <c r="AX1" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="AX1" s="1" t="s">
+      <c r="AY1" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="AY1" s="1" t="s">
+      <c r="AZ1" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="AZ1" s="1" t="s">
+      <c r="BA1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="BA1" s="1" t="s">
+      <c r="BB1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="BB1" s="1" t="s">
+      <c r="BC1" s="1" t="s">
         <v>91</v>
-      </c>
-      <c r="BC1" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="BD1" s="1" t="s">
-        <v>93</v>
       </c>
     </row>
   </sheetData>
@@ -1091,7 +1076,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6286078E-1D16-4E4D-BF5F-BEF494AF7186}">
-  <dimension ref="A1:N25"/>
+  <dimension ref="A1:N24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29.28515625" bestFit="1" customWidth="1"/>
@@ -1296,11 +1281,6 @@
         <v>36</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>37</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>